<commit_message>
新增 memories 和 contracts 表，events 加 contract_code 字段
</commit_message>
<xml_diff>
--- a/readme/ai驱动针织面料贸易软件erp设计_4.xlsx
+++ b/readme/ai驱动针织面料贸易软件erp设计_4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicjiang/aierp/开发文档/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicjiang/aierp/readme/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2DCA59-FB7E-4F4F-8450-4409EF9C47E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B602F5A-0255-4F4A-85ED-CF86BAEDEA3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="25880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -645,6 +645,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>656089</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>131217</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>614381</xdr:colOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>82713</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图形 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{324FAE78-E97E-8AAB-0E9A-BC33CB5A3F00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="656089" y="22869372"/>
+          <a:ext cx="6477000" cy="7810500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1715,5 +1770,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>